<commit_message>
Add support for image process on JavaScript side (#902)
</commit_message>
<xml_diff>
--- a/zigar-compiler/test/integration/test-matrix.xlsx
+++ b/zigar-compiler/test/integration/test-matrix.xlsx
@@ -18,24 +18,25 @@
     <sheet name="Thread handling" sheetId="8" r:id="rId11"/>
     <sheet name="Package manager" sheetId="9" r:id="rId12"/>
     <sheet name="Iterator" sheetId="10" r:id="rId13"/>
-    <sheet name="Stream handling" sheetId="11" r:id="rId14"/>
-    <sheet name="Metadata" sheetId="12" r:id="rId15"/>
-    <sheet name="Options" sheetId="13" r:id="rId16"/>
+    <sheet name="Image processing" sheetId="11" r:id="rId14"/>
+    <sheet name="Stream handling" sheetId="12" r:id="rId15"/>
+    <sheet name="Metadata" sheetId="13" r:id="rId16"/>
+    <sheet name="Options" sheetId="14" r:id="rId17"/>
   </sheets>
   <calcPr iterateDelta="0.0001"/>
   <extLst>
     <ext uri="smNativeData">
-      <pm:revision xmlns:pm="smNativeData" day="1778697221" val="1234" rev="124" rev64="64" revOS="3" revMin="124" revMax="0"/>
-      <pm:docPrefs xmlns:pm="smNativeData" id="1778697221" fixedDigits="0" showNotice="1" showFrameBounds="1" autoChart="1" recalcOnPrint="1" recalcOnCopy="1" finalRounding="1" compatTextArt="1" tab="567" useDefinedPrintRange="1" printArea="currentSheet"/>
-      <pm:compatibility xmlns:pm="smNativeData" id="1778697221" overlapCells="1"/>
-      <pm:defCurrency xmlns:pm="smNativeData" id="1778697221"/>
+      <pm:revision xmlns:pm="smNativeData" day="1782245724" val="1234" rev="124" rev64="64" revOS="3" revMin="124" revMax="0"/>
+      <pm:docPrefs xmlns:pm="smNativeData" id="1782245724" fixedDigits="0" showNotice="1" showFrameBounds="1" autoChart="1" recalcOnPrint="1" recalcOnCopy="1" finalRounding="1" compatTextArt="1" tab="567" useDefinedPrintRange="1" printArea="currentSheet"/>
+      <pm:compatibility xmlns:pm="smNativeData" id="1782245724" overlapCells="1"/>
+      <pm:defCurrency xmlns:pm="smNativeData" id="1782245724"/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="680" uniqueCount="234">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="713" uniqueCount="250">
   <si>
     <t>Context</t>
   </si>
@@ -370,6 +371,30 @@
     <t>std.fs.path.ComponentIterator</t>
   </si>
   <si>
+    <t>Basic rendering</t>
+  </si>
+  <si>
+    <t>Resizing</t>
+  </si>
+  <si>
+    <t>Sepia</t>
+  </si>
+  <si>
+    <t>Circle pattern</t>
+  </si>
+  <si>
+    <t>Metallic</t>
+  </si>
+  <si>
+    <t>Droste</t>
+  </si>
+  <si>
+    <t>Raytracing</t>
+  </si>
+  <si>
+    <t>Mandelbulb</t>
+  </si>
+  <si>
     <t>Read from file</t>
   </si>
   <si>
@@ -698,6 +723,30 @@
   </si>
   <si>
     <t>Copy virtual file to real file using sendfile</t>
+  </si>
+  <si>
+    <t>Get file descriptor using libc function</t>
+  </si>
+  <si>
+    <t>Check if stream is terminal using libc function</t>
+  </si>
+  <si>
+    <t>Get terminal name using libc function</t>
+  </si>
+  <si>
+    <t>Truncate file using posix function</t>
+  </si>
+  <si>
+    <t>Truncate opened file using posix function</t>
+  </si>
+  <si>
+    <t>Truncate opened file using win32 function</t>
+  </si>
+  <si>
+    <t>Copy real file to virtual file using copy_file_range</t>
+  </si>
+  <si>
+    <t>Copy virtual file to real file file using copy_file_range</t>
   </si>
   <si>
     <t>Field as string</t>
@@ -766,7 +815,7 @@
       <sz val="11"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1778697221" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1782245724" ulstyle="none" kern="1">
             <pm:latin face="Calibri" sz="220" lang="default"/>
             <pm:cs face="Basic Roman" sz="220" lang="default"/>
             <pm:ea face="Basic Roman" sz="220" lang="default"/>
@@ -781,7 +830,7 @@
       <sz val="10"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1778697221" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1782245724" ulstyle="none" kern="1">
             <pm:latin face="Basic Sans" sz="200" lang="default"/>
             <pm:cs face="Basic Roman" sz="200" lang="default"/>
             <pm:ea face="Basic Roman" sz="200" lang="default"/>
@@ -796,7 +845,7 @@
       <sz val="10"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1778697221" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1782245724" ulstyle="none" kern="1">
             <pm:latin face="Arial" sz="200" lang="default"/>
             <pm:cs face="Basic Roman" sz="200" lang="default"/>
             <pm:ea face="Basic Roman" sz="200" lang="default"/>
@@ -812,7 +861,7 @@
       <sz val="11"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1778697221" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1782245724" ulstyle="none" kern="1">
             <pm:latin face="Calibri" sz="220" lang="default" weight="bold"/>
             <pm:cs face="Basic Roman" sz="220" lang="default" weight="bold"/>
             <pm:ea face="Basic Roman" sz="220" lang="default" weight="bold"/>
@@ -821,7 +870,7 @@
       </extLst>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -834,7 +883,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1778697221" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
+            <pm:shade xmlns:pm="smNativeData" id="1782245724" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
           </ext>
         </extLst>
       </patternFill>
@@ -845,7 +894,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1778697221" type="1" fgLvl="100" fgClr="0081D41A" bgLvl="0" bgClr="0092D050"/>
+            <pm:shade xmlns:pm="smNativeData" id="1782245724" type="1" fgLvl="100" fgClr="0081D41A" bgLvl="0" bgClr="0092D050"/>
           </ext>
         </extLst>
       </patternFill>
@@ -856,7 +905,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1778697221" type="1" fgLvl="100" fgClr="0092D050" bgLvl="0" bgClr="0081D41A"/>
+            <pm:shade xmlns:pm="smNativeData" id="1782245724" type="1" fgLvl="100" fgClr="0092D050" bgLvl="0" bgClr="0081D41A"/>
           </ext>
         </extLst>
       </patternFill>
@@ -867,7 +916,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1778697221" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
+            <pm:shade xmlns:pm="smNativeData" id="1782245724" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
           </ext>
         </extLst>
       </patternFill>
@@ -878,35 +927,13 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1778697221" type="1" fgLvl="100" fgClr="00999999" bgLvl="0" bgClr="00808080"/>
-          </ext>
-        </extLst>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFFF"/>
-        <bgColor rgb="FFFFFFFF"/>
-        <extLst>
-          <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1778697221" type="1" fgLvl="100" fgClr="00FFFFFF" bgLvl="100" bgClr="00000000"/>
-          </ext>
-        </extLst>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC000"/>
-        <bgColor rgb="FFFFFFFF"/>
-        <extLst>
-          <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1778697221" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
+            <pm:shade xmlns:pm="smNativeData" id="1782245724" type="1" fgLvl="100" fgClr="00999999" bgLvl="0" bgClr="00808080"/>
           </ext>
         </extLst>
       </patternFill>
     </fill>
   </fills>
-  <borders count="8">
+  <borders count="6">
     <border>
       <left style="none">
         <color rgb="FF000000"/>
@@ -922,7 +949,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1778697221"/>
+          <pm:border xmlns:pm="smNativeData" id="1782245724"/>
         </ext>
       </extLst>
     </border>
@@ -941,7 +968,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1778697221">
+          <pm:border xmlns:pm="smNativeData" id="1782245724">
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="right" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
           </pm:border>
@@ -963,7 +990,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1778697221">
+          <pm:border xmlns:pm="smNativeData" id="1782245724">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -987,7 +1014,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1778697221">
+          <pm:border xmlns:pm="smNativeData" id="1782245724">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -1011,7 +1038,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1778697221">
+          <pm:border xmlns:pm="smNativeData" id="1782245724">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -1035,45 +1062,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1778697221"/>
-        </ext>
-      </extLst>
-    </border>
-    <border>
-      <left style="none">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="none">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="none">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="none">
-        <color rgb="FF000000"/>
-      </bottom>
-      <extLst>
-        <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1778697221"/>
-        </ext>
-      </extLst>
-    </border>
-    <border>
-      <left style="none">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="none">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="none">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="none">
-        <color rgb="FF000000"/>
-      </bottom>
-      <extLst>
-        <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1778697221"/>
+          <pm:border xmlns:pm="smNativeData" id="1782245724"/>
         </ext>
       </extLst>
     </border>
@@ -1123,13 +1112,13 @@
     <cellStyle name="Currency [0]" xfId="4" builtinId="7" customBuiltin="1"/>
     <cellStyle name="Percent" xfId="5" builtinId="5" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="13">
+  <dxfs count="15">
     <dxf>
       <font>
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778697221" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1782245724" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1142,7 +1131,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778697221" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1782245724" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1153,7 +1142,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778697221" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1782245724" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1166,7 +1155,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778697221" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1782245724" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1177,7 +1166,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778697221" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1782245724" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1190,7 +1179,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778697221" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1782245724" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1201,7 +1190,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778697221" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1782245724" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1214,7 +1203,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778697221" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1782245724" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1225,7 +1214,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778697221" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1782245724" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1238,7 +1227,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778697221" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1782245724" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1249,7 +1238,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778697221" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1782245724" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1262,7 +1251,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778697221" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1782245724" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1273,7 +1262,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778697221" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1782245724" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1286,7 +1275,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778697221" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1782245724" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1297,7 +1286,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778697221" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1782245724" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1310,7 +1299,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778697221" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1782245724" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1321,7 +1310,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778697221" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1782245724" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1334,7 +1323,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778697221" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1782245724" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1345,7 +1334,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778697221" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1782245724" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1358,7 +1347,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778697221" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1782245724" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1369,7 +1358,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778697221" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1782245724" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1382,7 +1371,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778697221" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1782245724" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1393,7 +1382,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778697221" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1782245724" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1406,7 +1395,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778697221" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1782245724" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1417,7 +1406,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1778697221" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1782245724" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1430,7 +1419,55 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1778697221" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1782245724" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+            </ext>
+          </extLst>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+        <extLst>
+          <ext uri="smNativeData">
+            <pm:charSpec xmlns:pm="smNativeData" id="1782245724" fgClr="FF0000">
+              <pm:latin/>
+              <pm:cs/>
+              <pm:ea/>
+            </pm:charSpec>
+          </ext>
+        </extLst>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFB3B3"/>
+          <extLst>
+            <ext uri="smNativeData">
+              <pm:shade xmlns:pm="smNativeData" id="1782245724" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+            </ext>
+          </extLst>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+        <extLst>
+          <ext uri="smNativeData">
+            <pm:charSpec xmlns:pm="smNativeData" id="1782245724" fgClr="FF0000">
+              <pm:latin/>
+              <pm:cs/>
+              <pm:ea/>
+            </pm:charSpec>
+          </ext>
+        </extLst>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFB3B3"/>
+          <extLst>
+            <ext uri="smNativeData">
+              <pm:shade xmlns:pm="smNativeData" id="1782245724" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1440,10 +1477,10 @@
   <tableStyles count="0"/>
   <extLst>
     <ext uri="smNativeData">
-      <pm:charStyles xmlns:pm="smNativeData" id="1778697221" count="1">
+      <pm:charStyles xmlns:pm="smNativeData" id="1782245724" count="1">
         <pm:charStyle name="Normal" fontId="0" Id="1"/>
       </pm:charStyles>
-      <pm:colors xmlns:pm="smNativeData" id="1778697221" count="6">
+      <pm:colors xmlns:pm="smNativeData" id="1782245724" count="6">
         <pm:color name="Color 24" rgb="FFC000"/>
         <pm:color name="Color 25" rgb="FF9900"/>
         <pm:color name="Color 26" rgb="81D41A"/>
@@ -2747,7 +2784,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778697221" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1782245724" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -2756,14 +2793,14 @@
   <headerFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778697221" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778697221" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1782245724" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1782245724" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778697221" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1782245724" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -2843,7 +2880,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778697221" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1782245724" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -2854,14 +2891,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778697221" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778697221" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1782245724" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1782245724" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778697221" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1782245724" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -2872,7 +2909,133 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <dimension ref="A1:D112"/>
+  <dimension ref="A1:B10"/>
+  <sheetFormatPr baseColWidth="9" defaultColWidth="10.000000" defaultRowHeight="15.40"/>
+  <cols>
+    <col min="1" max="1" width="32.901786" customWidth="1"/>
+    <col min="2" max="2" width="9.330357" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="B1" s="12"/>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" s="6"/>
+      <c r="B2" s="12"/>
+    </row>
+    <row r="3" spans="1:2">
+      <c r="A3" s="9" t="s">
+        <v>111</v>
+      </c>
+      <c r="B3" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
+      <c r="A4" s="9" t="s">
+        <v>112</v>
+      </c>
+      <c r="B4" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2">
+      <c r="A5" s="9" t="s">
+        <v>113</v>
+      </c>
+      <c r="B5" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2">
+      <c r="A6" s="9" t="s">
+        <v>114</v>
+      </c>
+      <c r="B6" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2">
+      <c r="A7" s="9" t="s">
+        <v>115</v>
+      </c>
+      <c r="B7" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2">
+      <c r="A8" s="9" t="s">
+        <v>116</v>
+      </c>
+      <c r="B8" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2">
+      <c r="A9" s="9" t="s">
+        <v>117</v>
+      </c>
+      <c r="B9" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2">
+      <c r="A10" s="9" t="s">
+        <v>118</v>
+      </c>
+      <c r="B10" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="B1:B2"/>
+  </mergeCells>
+  <conditionalFormatting sqref="B3:B10">
+    <cfRule type="cellIs" dxfId="10" priority="1" operator="equal">
+      <formula>"N"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B3:B10">
+    <cfRule type="cellIs" dxfId="11" priority="2" operator="equal">
+      <formula>#NAME?</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <printOptions>
+    <extLst>
+      <ext uri="smNativeData">
+        <pm:pageFlags xmlns:pm="smNativeData" id="1782245724" printRowHead="0" printColHead="0" printHeadLine="0" printFootLine="0" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+      </ext>
+    </extLst>
+  </printOptions>
+  <pageMargins left="1.000000" right="1.000000" top="1.000000" bottom="1.000000" header="0.393750" footer="0.393750"/>
+  <pageSetup paperSize="1" fitToWidth="0" fitToHeight="1" pageOrder="overThenDown"/>
+  <headerFooter>
+    <extLst>
+      <ext uri="smNativeData">
+        <pm:header xmlns:pm="smNativeData" id="1782245724" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1782245724" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+      </ext>
+    </extLst>
+  </headerFooter>
+  <extLst>
+    <ext uri="smNativeData">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1782245724" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+        <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
+        <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
+      </pm:sheetPrefs>
+    </ext>
+  </extLst>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <dimension ref="A1:D120"/>
   <sheetFormatPr defaultRowHeight="15.40"/>
   <cols>
     <col min="1" max="1" width="62.312500" customWidth="1" style="0"/>
@@ -2891,7 +3054,7 @@
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="9" t="s">
-        <v>111</v>
+        <v>119</v>
       </c>
       <c r="B3" s="10" t="s">
         <v>26</v>
@@ -2900,7 +3063,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="B4" s="10" t="s">
         <v>26</v>
@@ -2908,7 +3071,7 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="B5" s="10" t="s">
         <v>26</v>
@@ -2916,7 +3079,7 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="9" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="B6" s="10" t="s">
         <v>26</v>
@@ -2924,7 +3087,7 @@
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="9" t="s">
-        <v>115</v>
+        <v>123</v>
       </c>
       <c r="B7" s="10" t="s">
         <v>26</v>
@@ -2932,7 +3095,7 @@
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="9" t="s">
-        <v>116</v>
+        <v>124</v>
       </c>
       <c r="B8" s="10" t="s">
         <v>26</v>
@@ -2940,7 +3103,7 @@
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="9" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
       <c r="B9" s="10" t="s">
         <v>26</v>
@@ -2948,7 +3111,7 @@
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="9" t="s">
-        <v>118</v>
+        <v>126</v>
       </c>
       <c r="B10" s="10" t="s">
         <v>26</v>
@@ -2956,7 +3119,7 @@
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="9" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="B11" s="10" t="s">
         <v>26</v>
@@ -2964,7 +3127,7 @@
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="9" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
       <c r="B12" s="10" t="s">
         <v>26</v>
@@ -2972,7 +3135,7 @@
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="9" t="s">
-        <v>121</v>
+        <v>129</v>
       </c>
       <c r="B13" s="10" t="s">
         <v>26</v>
@@ -2980,7 +3143,7 @@
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="9" t="s">
-        <v>122</v>
+        <v>130</v>
       </c>
       <c r="B14" s="10" t="s">
         <v>26</v>
@@ -2988,7 +3151,7 @@
     </row>
     <row r="15" spans="1:2">
       <c r="A15" s="9" t="s">
-        <v>123</v>
+        <v>131</v>
       </c>
       <c r="B15" s="10" t="s">
         <v>26</v>
@@ -2996,7 +3159,7 @@
     </row>
     <row r="16" spans="1:2">
       <c r="A16" s="9" t="s">
-        <v>124</v>
+        <v>132</v>
       </c>
       <c r="B16" s="10" t="s">
         <v>26</v>
@@ -3004,7 +3167,7 @@
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="9" t="s">
-        <v>125</v>
+        <v>133</v>
       </c>
       <c r="B17" s="10" t="s">
         <v>26</v>
@@ -3012,7 +3175,7 @@
     </row>
     <row r="18" spans="1:2">
       <c r="A18" s="9" t="s">
-        <v>126</v>
+        <v>134</v>
       </c>
       <c r="B18" s="10" t="s">
         <v>26</v>
@@ -3020,7 +3183,7 @@
     </row>
     <row r="19" spans="1:2">
       <c r="A19" s="9" t="s">
-        <v>127</v>
+        <v>135</v>
       </c>
       <c r="B19" s="10" t="s">
         <v>26</v>
@@ -3028,7 +3191,7 @@
     </row>
     <row r="20" spans="1:2">
       <c r="A20" s="9" t="s">
-        <v>128</v>
+        <v>136</v>
       </c>
       <c r="B20" s="10" t="s">
         <v>26</v>
@@ -3036,7 +3199,7 @@
     </row>
     <row r="21" spans="1:2">
       <c r="A21" s="9" t="s">
-        <v>129</v>
+        <v>137</v>
       </c>
       <c r="B21" s="10" t="s">
         <v>26</v>
@@ -3044,7 +3207,7 @@
     </row>
     <row r="22" spans="1:2">
       <c r="A22" s="9" t="s">
-        <v>130</v>
+        <v>138</v>
       </c>
       <c r="B22" s="10" t="s">
         <v>26</v>
@@ -3052,7 +3215,7 @@
     </row>
     <row r="23" spans="1:2">
       <c r="A23" s="9" t="s">
-        <v>131</v>
+        <v>139</v>
       </c>
       <c r="B23" s="10" t="s">
         <v>26</v>
@@ -3060,7 +3223,7 @@
     </row>
     <row r="24" spans="1:2">
       <c r="A24" s="9" t="s">
-        <v>132</v>
+        <v>140</v>
       </c>
       <c r="B24" s="10" t="s">
         <v>26</v>
@@ -3068,7 +3231,7 @@
     </row>
     <row r="25" spans="1:2">
       <c r="A25" s="9" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="B25" s="10" t="s">
         <v>26</v>
@@ -3076,7 +3239,7 @@
     </row>
     <row r="26" spans="1:2">
       <c r="A26" s="9" t="s">
-        <v>134</v>
+        <v>142</v>
       </c>
       <c r="B26" s="10" t="s">
         <v>26</v>
@@ -3084,7 +3247,7 @@
     </row>
     <row r="27" spans="1:2">
       <c r="A27" s="9" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="B27" s="10" t="s">
         <v>26</v>
@@ -3092,7 +3255,7 @@
     </row>
     <row r="28" spans="1:2">
       <c r="A28" s="9" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="B28" s="10" t="s">
         <v>26</v>
@@ -3100,7 +3263,7 @@
     </row>
     <row r="29" spans="1:2">
       <c r="A29" s="9" t="s">
-        <v>137</v>
+        <v>145</v>
       </c>
       <c r="B29" s="10" t="s">
         <v>26</v>
@@ -3108,7 +3271,7 @@
     </row>
     <row r="30" spans="1:2">
       <c r="A30" s="9" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
       <c r="B30" s="10" t="s">
         <v>26</v>
@@ -3116,7 +3279,7 @@
     </row>
     <row r="31" spans="1:2">
       <c r="A31" s="9" t="s">
-        <v>139</v>
+        <v>147</v>
       </c>
       <c r="B31" s="10" t="s">
         <v>26</v>
@@ -3124,7 +3287,7 @@
     </row>
     <row r="32" spans="1:2">
       <c r="A32" s="9" t="s">
-        <v>140</v>
+        <v>148</v>
       </c>
       <c r="B32" s="10" t="s">
         <v>26</v>
@@ -3132,7 +3295,7 @@
     </row>
     <row r="33" spans="1:2">
       <c r="A33" s="9" t="s">
-        <v>141</v>
+        <v>149</v>
       </c>
       <c r="B33" s="10" t="s">
         <v>26</v>
@@ -3140,7 +3303,7 @@
     </row>
     <row r="34" spans="1:2">
       <c r="A34" s="9" t="s">
-        <v>142</v>
+        <v>150</v>
       </c>
       <c r="B34" s="10" t="s">
         <v>26</v>
@@ -3148,7 +3311,7 @@
     </row>
     <row r="35" spans="1:2">
       <c r="A35" s="9" t="s">
-        <v>143</v>
+        <v>151</v>
       </c>
       <c r="B35" s="10" t="s">
         <v>26</v>
@@ -3156,7 +3319,7 @@
     </row>
     <row r="36" spans="1:2">
       <c r="A36" s="9" t="s">
-        <v>144</v>
+        <v>152</v>
       </c>
       <c r="B36" s="10" t="s">
         <v>26</v>
@@ -3164,7 +3327,7 @@
     </row>
     <row r="37" spans="1:2">
       <c r="A37" s="9" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="B37" s="10" t="s">
         <v>26</v>
@@ -3172,7 +3335,7 @@
     </row>
     <row r="38" spans="1:2">
       <c r="A38" s="9" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="B38" s="10" t="s">
         <v>26</v>
@@ -3180,7 +3343,7 @@
     </row>
     <row r="39" spans="1:2">
       <c r="A39" s="9" t="s">
-        <v>147</v>
+        <v>155</v>
       </c>
       <c r="B39" s="10" t="s">
         <v>26</v>
@@ -3188,7 +3351,7 @@
     </row>
     <row r="40" spans="1:2">
       <c r="A40" s="9" t="s">
-        <v>148</v>
+        <v>156</v>
       </c>
       <c r="B40" s="10" t="s">
         <v>26</v>
@@ -3196,7 +3359,7 @@
     </row>
     <row r="41" spans="1:2">
       <c r="A41" s="9" t="s">
-        <v>149</v>
+        <v>157</v>
       </c>
       <c r="B41" s="10" t="s">
         <v>26</v>
@@ -3204,7 +3367,7 @@
     </row>
     <row r="42" spans="1:2">
       <c r="A42" s="9" t="s">
-        <v>150</v>
+        <v>158</v>
       </c>
       <c r="B42" s="10" t="s">
         <v>26</v>
@@ -3212,7 +3375,7 @@
     </row>
     <row r="43" spans="1:2">
       <c r="A43" s="9" t="s">
-        <v>151</v>
+        <v>159</v>
       </c>
       <c r="B43" s="10" t="s">
         <v>26</v>
@@ -3220,7 +3383,7 @@
     </row>
     <row r="44" spans="1:2">
       <c r="A44" s="9" t="s">
-        <v>152</v>
+        <v>160</v>
       </c>
       <c r="B44" s="10" t="s">
         <v>26</v>
@@ -3228,7 +3391,7 @@
     </row>
     <row r="45" spans="1:2">
       <c r="A45" s="9" t="s">
-        <v>153</v>
+        <v>161</v>
       </c>
       <c r="B45" s="10" t="s">
         <v>26</v>
@@ -3236,7 +3399,7 @@
     </row>
     <row r="46" spans="1:2">
       <c r="A46" s="9" t="s">
-        <v>154</v>
+        <v>162</v>
       </c>
       <c r="B46" s="10" t="s">
         <v>26</v>
@@ -3244,7 +3407,7 @@
     </row>
     <row r="47" spans="1:2">
       <c r="A47" s="9" t="s">
-        <v>155</v>
+        <v>163</v>
       </c>
       <c r="B47" s="10" t="s">
         <v>26</v>
@@ -3252,7 +3415,7 @@
     </row>
     <row r="48" spans="1:2">
       <c r="A48" s="9" t="s">
-        <v>156</v>
+        <v>164</v>
       </c>
       <c r="B48" s="10" t="s">
         <v>26</v>
@@ -3260,7 +3423,7 @@
     </row>
     <row r="49" spans="1:2">
       <c r="A49" s="9" t="s">
-        <v>157</v>
+        <v>165</v>
       </c>
       <c r="B49" s="10" t="s">
         <v>26</v>
@@ -3268,7 +3431,7 @@
     </row>
     <row r="50" spans="1:2">
       <c r="A50" s="9" t="s">
-        <v>158</v>
+        <v>166</v>
       </c>
       <c r="B50" s="10" t="s">
         <v>26</v>
@@ -3276,7 +3439,7 @@
     </row>
     <row r="51" spans="1:2">
       <c r="A51" s="9" t="s">
-        <v>159</v>
+        <v>167</v>
       </c>
       <c r="B51" s="10" t="s">
         <v>26</v>
@@ -3284,7 +3447,7 @@
     </row>
     <row r="52" spans="1:2">
       <c r="A52" s="9" t="s">
-        <v>160</v>
+        <v>168</v>
       </c>
       <c r="B52" s="10" t="s">
         <v>26</v>
@@ -3292,7 +3455,7 @@
     </row>
     <row r="53" spans="1:2">
       <c r="A53" s="9" t="s">
-        <v>161</v>
+        <v>169</v>
       </c>
       <c r="B53" s="10" t="s">
         <v>26</v>
@@ -3300,7 +3463,7 @@
     </row>
     <row r="54" spans="1:2">
       <c r="A54" s="9" t="s">
-        <v>162</v>
+        <v>170</v>
       </c>
       <c r="B54" s="10" t="s">
         <v>26</v>
@@ -3308,7 +3471,7 @@
     </row>
     <row r="55" spans="1:2">
       <c r="A55" s="9" t="s">
-        <v>163</v>
+        <v>171</v>
       </c>
       <c r="B55" s="10" t="s">
         <v>26</v>
@@ -3316,7 +3479,7 @@
     </row>
     <row r="56" spans="1:2">
       <c r="A56" s="9" t="s">
-        <v>164</v>
+        <v>172</v>
       </c>
       <c r="B56" s="10" t="s">
         <v>26</v>
@@ -3324,7 +3487,7 @@
     </row>
     <row r="57" spans="1:2">
       <c r="A57" s="9" t="s">
-        <v>165</v>
+        <v>173</v>
       </c>
       <c r="B57" s="10" t="s">
         <v>26</v>
@@ -3332,7 +3495,7 @@
     </row>
     <row r="58" spans="1:2">
       <c r="A58" s="9" t="s">
-        <v>166</v>
+        <v>174</v>
       </c>
       <c r="B58" s="10" t="s">
         <v>26</v>
@@ -3340,7 +3503,7 @@
     </row>
     <row r="59" spans="1:2">
       <c r="A59" s="9" t="s">
-        <v>167</v>
+        <v>175</v>
       </c>
       <c r="B59" s="10" t="s">
         <v>26</v>
@@ -3348,7 +3511,7 @@
     </row>
     <row r="60" spans="1:2">
       <c r="A60" s="9" t="s">
-        <v>168</v>
+        <v>176</v>
       </c>
       <c r="B60" s="10" t="s">
         <v>26</v>
@@ -3356,7 +3519,7 @@
     </row>
     <row r="61" spans="1:2">
       <c r="A61" s="9" t="s">
-        <v>169</v>
+        <v>177</v>
       </c>
       <c r="B61" s="10" t="s">
         <v>26</v>
@@ -3364,7 +3527,7 @@
     </row>
     <row r="62" spans="1:2">
       <c r="A62" s="9" t="s">
-        <v>170</v>
+        <v>178</v>
       </c>
       <c r="B62" s="10" t="s">
         <v>26</v>
@@ -3372,7 +3535,7 @@
     </row>
     <row r="63" spans="1:2">
       <c r="A63" s="9" t="s">
-        <v>171</v>
+        <v>179</v>
       </c>
       <c r="B63" s="10" t="s">
         <v>26</v>
@@ -3380,7 +3543,7 @@
     </row>
     <row r="64" spans="1:2">
       <c r="A64" s="9" t="s">
-        <v>172</v>
+        <v>180</v>
       </c>
       <c r="B64" s="10" t="s">
         <v>26</v>
@@ -3388,7 +3551,7 @@
     </row>
     <row r="65" spans="1:2">
       <c r="A65" s="9" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="B65" s="10" t="s">
         <v>26</v>
@@ -3396,7 +3559,7 @@
     </row>
     <row r="66" spans="1:2">
       <c r="A66" s="9" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="B66" s="10" t="s">
         <v>26</v>
@@ -3404,7 +3567,7 @@
     </row>
     <row r="67" spans="1:2">
       <c r="A67" s="9" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
       <c r="B67" s="10" t="s">
         <v>26</v>
@@ -3412,7 +3575,7 @@
     </row>
     <row r="68" spans="1:2">
       <c r="A68" s="9" t="s">
-        <v>176</v>
+        <v>184</v>
       </c>
       <c r="B68" s="10" t="s">
         <v>26</v>
@@ -3420,7 +3583,7 @@
     </row>
     <row r="69" spans="1:2">
       <c r="A69" s="9" t="s">
-        <v>177</v>
+        <v>185</v>
       </c>
       <c r="B69" s="10" t="s">
         <v>26</v>
@@ -3428,7 +3591,7 @@
     </row>
     <row r="70" spans="1:2">
       <c r="A70" s="9" t="s">
-        <v>178</v>
+        <v>186</v>
       </c>
       <c r="B70" s="10" t="s">
         <v>26</v>
@@ -3436,7 +3599,7 @@
     </row>
     <row r="71" spans="1:2">
       <c r="A71" s="9" t="s">
-        <v>179</v>
+        <v>187</v>
       </c>
       <c r="B71" s="10" t="s">
         <v>26</v>
@@ -3444,7 +3607,7 @@
     </row>
     <row r="72" spans="1:2">
       <c r="A72" s="9" t="s">
-        <v>180</v>
+        <v>188</v>
       </c>
       <c r="B72" s="10" t="s">
         <v>26</v>
@@ -3452,7 +3615,7 @@
     </row>
     <row r="73" spans="1:2">
       <c r="A73" s="9" t="s">
-        <v>181</v>
+        <v>189</v>
       </c>
       <c r="B73" s="10" t="s">
         <v>26</v>
@@ -3460,7 +3623,7 @@
     </row>
     <row r="74" spans="1:2">
       <c r="A74" s="9" t="s">
-        <v>182</v>
+        <v>190</v>
       </c>
       <c r="B74" s="10" t="s">
         <v>26</v>
@@ -3468,7 +3631,7 @@
     </row>
     <row r="75" spans="1:2">
       <c r="A75" s="9" t="s">
-        <v>183</v>
+        <v>191</v>
       </c>
       <c r="B75" s="10" t="s">
         <v>26</v>
@@ -3476,7 +3639,7 @@
     </row>
     <row r="76" spans="1:2">
       <c r="A76" s="9" t="s">
-        <v>184</v>
+        <v>192</v>
       </c>
       <c r="B76" s="10" t="s">
         <v>26</v>
@@ -3484,7 +3647,7 @@
     </row>
     <row r="77" spans="1:2">
       <c r="A77" s="9" t="s">
-        <v>185</v>
+        <v>193</v>
       </c>
       <c r="B77" s="10" t="s">
         <v>26</v>
@@ -3492,7 +3655,7 @@
     </row>
     <row r="78" spans="1:2">
       <c r="A78" s="9" t="s">
-        <v>186</v>
+        <v>194</v>
       </c>
       <c r="B78" s="10" t="s">
         <v>26</v>
@@ -3500,7 +3663,7 @@
     </row>
     <row r="79" spans="1:2">
       <c r="A79" s="9" t="s">
-        <v>187</v>
+        <v>195</v>
       </c>
       <c r="B79" s="10" t="s">
         <v>26</v>
@@ -3508,7 +3671,7 @@
     </row>
     <row r="80" spans="1:2">
       <c r="A80" s="9" t="s">
-        <v>188</v>
+        <v>196</v>
       </c>
       <c r="B80" s="10" t="s">
         <v>26</v>
@@ -3516,7 +3679,7 @@
     </row>
     <row r="81" spans="1:2">
       <c r="A81" s="9" t="s">
-        <v>189</v>
+        <v>197</v>
       </c>
       <c r="B81" s="10" t="s">
         <v>26</v>
@@ -3524,7 +3687,7 @@
     </row>
     <row r="82" spans="1:2">
       <c r="A82" s="9" t="s">
-        <v>190</v>
+        <v>198</v>
       </c>
       <c r="B82" s="10" t="s">
         <v>26</v>
@@ -3532,7 +3695,7 @@
     </row>
     <row r="83" spans="1:2">
       <c r="A83" s="9" t="s">
-        <v>191</v>
+        <v>199</v>
       </c>
       <c r="B83" s="10" t="s">
         <v>26</v>
@@ -3540,7 +3703,7 @@
     </row>
     <row r="84" spans="1:2">
       <c r="A84" s="9" t="s">
-        <v>192</v>
+        <v>200</v>
       </c>
       <c r="B84" s="10" t="s">
         <v>26</v>
@@ -3548,7 +3711,7 @@
     </row>
     <row r="85" spans="1:2">
       <c r="A85" s="9" t="s">
-        <v>193</v>
+        <v>201</v>
       </c>
       <c r="B85" s="10" t="s">
         <v>26</v>
@@ -3556,7 +3719,7 @@
     </row>
     <row r="86" spans="1:2">
       <c r="A86" s="9" t="s">
-        <v>194</v>
+        <v>202</v>
       </c>
       <c r="B86" s="10" t="s">
         <v>26</v>
@@ -3564,7 +3727,7 @@
     </row>
     <row r="87" spans="1:2">
       <c r="A87" s="9" t="s">
-        <v>195</v>
+        <v>203</v>
       </c>
       <c r="B87" s="10" t="s">
         <v>26</v>
@@ -3572,7 +3735,7 @@
     </row>
     <row r="88" spans="1:2">
       <c r="A88" s="9" t="s">
-        <v>196</v>
+        <v>204</v>
       </c>
       <c r="B88" s="10" t="s">
         <v>26</v>
@@ -3580,7 +3743,7 @@
     </row>
     <row r="89" spans="1:2">
       <c r="A89" s="9" t="s">
-        <v>197</v>
+        <v>205</v>
       </c>
       <c r="B89" s="10" t="s">
         <v>26</v>
@@ -3588,7 +3751,7 @@
     </row>
     <row r="90" spans="1:2">
       <c r="A90" s="9" t="s">
-        <v>198</v>
+        <v>206</v>
       </c>
       <c r="B90" s="10" t="s">
         <v>26</v>
@@ -3596,7 +3759,7 @@
     </row>
     <row r="91" spans="1:2">
       <c r="A91" s="9" t="s">
-        <v>199</v>
+        <v>207</v>
       </c>
       <c r="B91" s="10" t="s">
         <v>26</v>
@@ -3604,7 +3767,7 @@
     </row>
     <row r="92" spans="1:2">
       <c r="A92" s="9" t="s">
-        <v>200</v>
+        <v>208</v>
       </c>
       <c r="B92" s="10" t="s">
         <v>26</v>
@@ -3612,7 +3775,7 @@
     </row>
     <row r="93" spans="1:2">
       <c r="A93" s="9" t="s">
-        <v>201</v>
+        <v>209</v>
       </c>
       <c r="B93" s="10" t="s">
         <v>26</v>
@@ -3620,7 +3783,7 @@
     </row>
     <row r="94" spans="1:2">
       <c r="A94" s="9" t="s">
-        <v>202</v>
+        <v>210</v>
       </c>
       <c r="B94" s="10" t="s">
         <v>26</v>
@@ -3628,7 +3791,7 @@
     </row>
     <row r="95" spans="1:2">
       <c r="A95" s="9" t="s">
-        <v>203</v>
+        <v>211</v>
       </c>
       <c r="B95" s="10" t="s">
         <v>26</v>
@@ -3636,7 +3799,7 @@
     </row>
     <row r="96" spans="1:2">
       <c r="A96" s="9" t="s">
-        <v>204</v>
+        <v>212</v>
       </c>
       <c r="B96" s="10" t="s">
         <v>26</v>
@@ -3644,7 +3807,7 @@
     </row>
     <row r="97" spans="1:2">
       <c r="A97" s="9" t="s">
-        <v>205</v>
+        <v>213</v>
       </c>
       <c r="B97" s="10" t="s">
         <v>26</v>
@@ -3652,7 +3815,7 @@
     </row>
     <row r="98" spans="1:2">
       <c r="A98" s="9" t="s">
-        <v>206</v>
+        <v>214</v>
       </c>
       <c r="B98" s="10" t="s">
         <v>26</v>
@@ -3660,7 +3823,7 @@
     </row>
     <row r="99" spans="1:2">
       <c r="A99" s="9" t="s">
-        <v>207</v>
+        <v>215</v>
       </c>
       <c r="B99" s="10" t="s">
         <v>26</v>
@@ -3668,7 +3831,7 @@
     </row>
     <row r="100" spans="1:2">
       <c r="A100" s="9" t="s">
-        <v>208</v>
+        <v>216</v>
       </c>
       <c r="B100" s="10" t="s">
         <v>26</v>
@@ -3676,7 +3839,7 @@
     </row>
     <row r="101" spans="1:2">
       <c r="A101" s="9" t="s">
-        <v>209</v>
+        <v>217</v>
       </c>
       <c r="B101" s="10" t="s">
         <v>26</v>
@@ -3684,7 +3847,7 @@
     </row>
     <row r="102" spans="1:2">
       <c r="A102" s="9" t="s">
-        <v>210</v>
+        <v>218</v>
       </c>
       <c r="B102" s="10" t="s">
         <v>26</v>
@@ -3692,7 +3855,7 @@
     </row>
     <row r="103" spans="1:2">
       <c r="A103" s="9" t="s">
-        <v>211</v>
+        <v>219</v>
       </c>
       <c r="B103" s="10" t="s">
         <v>26</v>
@@ -3700,7 +3863,7 @@
     </row>
     <row r="104" spans="1:2">
       <c r="A104" s="9" t="s">
-        <v>212</v>
+        <v>220</v>
       </c>
       <c r="B104" s="10" t="s">
         <v>26</v>
@@ -3708,7 +3871,7 @@
     </row>
     <row r="105" spans="1:2">
       <c r="A105" s="9" t="s">
-        <v>213</v>
+        <v>221</v>
       </c>
       <c r="B105" s="10" t="s">
         <v>26</v>
@@ -3716,7 +3879,7 @@
     </row>
     <row r="106" spans="1:2">
       <c r="A106" s="9" t="s">
-        <v>214</v>
+        <v>222</v>
       </c>
       <c r="B106" s="10" t="s">
         <v>26</v>
@@ -3724,7 +3887,7 @@
     </row>
     <row r="107" spans="1:2">
       <c r="A107" s="9" t="s">
-        <v>215</v>
+        <v>223</v>
       </c>
       <c r="B107" s="10" t="s">
         <v>26</v>
@@ -3732,7 +3895,7 @@
     </row>
     <row r="108" spans="1:2">
       <c r="A108" s="9" t="s">
-        <v>216</v>
+        <v>224</v>
       </c>
       <c r="B108" s="10" t="s">
         <v>26</v>
@@ -3740,7 +3903,7 @@
     </row>
     <row r="109" spans="1:2">
       <c r="A109" s="9" t="s">
-        <v>217</v>
+        <v>225</v>
       </c>
       <c r="B109" s="10" t="s">
         <v>26</v>
@@ -3748,7 +3911,7 @@
     </row>
     <row r="110" spans="1:2">
       <c r="A110" s="9" t="s">
-        <v>218</v>
+        <v>226</v>
       </c>
       <c r="B110" s="10" t="s">
         <v>26</v>
@@ -3756,7 +3919,7 @@
     </row>
     <row r="111" spans="1:2">
       <c r="A111" s="9" t="s">
-        <v>219</v>
+        <v>227</v>
       </c>
       <c r="B111" s="10" t="s">
         <v>26</v>
@@ -3764,9 +3927,73 @@
     </row>
     <row r="112" spans="1:2">
       <c r="A112" s="9" t="s">
-        <v>220</v>
+        <v>228</v>
       </c>
       <c r="B112" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="113" spans="1:2">
+      <c r="A113" s="9" t="s">
+        <v>229</v>
+      </c>
+      <c r="B113" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="114" spans="1:2">
+      <c r="A114" s="9" t="s">
+        <v>230</v>
+      </c>
+      <c r="B114" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="115" spans="1:2">
+      <c r="A115" s="9" t="s">
+        <v>231</v>
+      </c>
+      <c r="B115" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="116" spans="1:2">
+      <c r="A116" s="9" t="s">
+        <v>232</v>
+      </c>
+      <c r="B116" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="117" spans="1:2">
+      <c r="A117" s="9" t="s">
+        <v>233</v>
+      </c>
+      <c r="B117" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="118" spans="1:2">
+      <c r="A118" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="B118" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="119" spans="1:2">
+      <c r="A119" s="9" t="s">
+        <v>235</v>
+      </c>
+      <c r="B119" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="120" spans="1:2">
+      <c r="A120" s="9" t="s">
+        <v>236</v>
+      </c>
+      <c r="B120" s="10" t="s">
         <v>26</v>
       </c>
     </row>
@@ -3775,15 +4002,15 @@
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="B1:B2"/>
   </mergeCells>
-  <conditionalFormatting sqref="B3:B112">
-    <cfRule type="cellIs" dxfId="10" priority="1" operator="equal">
+  <conditionalFormatting sqref="B3:B120">
+    <cfRule type="cellIs" dxfId="12" priority="1" operator="equal">
       <formula>"N"</formula>
     </cfRule>
   </conditionalFormatting>
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778697221" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1782245724" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3794,14 +4021,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778697221" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778697221" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1782245724" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1782245724" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778697221" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1782245724" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3810,7 +4037,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <dimension ref="A1:B11"/>
   <sheetFormatPr defaultRowHeight="15.40"/>
@@ -3830,7 +4057,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>221</v>
+        <v>237</v>
       </c>
       <c r="B3" s="10" t="s">
         <v>26</v>
@@ -3838,7 +4065,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>222</v>
+        <v>238</v>
       </c>
       <c r="B4" s="10" t="s">
         <v>26</v>
@@ -3846,7 +4073,7 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
-        <v>223</v>
+        <v>239</v>
       </c>
       <c r="B5" s="10" t="s">
         <v>26</v>
@@ -3854,7 +4081,7 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="9" t="s">
-        <v>224</v>
+        <v>240</v>
       </c>
       <c r="B6" s="10" t="s">
         <v>26</v>
@@ -3862,7 +4089,7 @@
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="9" t="s">
-        <v>225</v>
+        <v>241</v>
       </c>
       <c r="B7" s="10" t="s">
         <v>26</v>
@@ -3870,15 +4097,15 @@
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="9" t="s">
-        <v>226</v>
+        <v>242</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>227</v>
+        <v>243</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="9" t="s">
-        <v>228</v>
+        <v>244</v>
       </c>
       <c r="B9" s="10" t="s">
         <v>26</v>
@@ -3886,7 +4113,7 @@
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="9" t="s">
-        <v>229</v>
+        <v>245</v>
       </c>
       <c r="B10" s="10" t="s">
         <v>26</v>
@@ -3894,7 +4121,7 @@
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="9" t="s">
-        <v>230</v>
+        <v>246</v>
       </c>
       <c r="B11" s="10" t="s">
         <v>26</v>
@@ -3906,14 +4133,14 @@
     <mergeCell ref="B1:B2"/>
   </mergeCells>
   <conditionalFormatting sqref="B3:B11">
-    <cfRule type="cellIs" dxfId="11" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="13" priority="1" operator="equal">
       <formula>"N"</formula>
     </cfRule>
   </conditionalFormatting>
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778697221" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1782245724" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3924,14 +4151,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778697221" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778697221" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1782245724" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1782245724" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778697221" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1782245724" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3940,7 +4167,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <dimension ref="A1:B5"/>
   <sheetFormatPr defaultRowHeight="15.40"/>
@@ -3960,7 +4187,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>231</v>
+        <v>247</v>
       </c>
       <c r="B3" s="10" t="s">
         <v>26</v>
@@ -3968,7 +4195,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>232</v>
+        <v>248</v>
       </c>
       <c r="B4" s="10" t="s">
         <v>26</v>
@@ -3976,7 +4203,7 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
-        <v>233</v>
+        <v>249</v>
       </c>
       <c r="B5" s="10" t="s">
         <v>26</v>
@@ -3988,14 +4215,14 @@
     <mergeCell ref="B1:B2"/>
   </mergeCells>
   <conditionalFormatting sqref="B3:B5">
-    <cfRule type="cellIs" dxfId="12" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="14" priority="1" operator="equal">
       <formula>"N"</formula>
     </cfRule>
   </conditionalFormatting>
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778697221" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1782245724" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -4006,14 +4233,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778697221" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778697221" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1782245724" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1782245724" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778697221" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1782245724" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -4069,7 +4296,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778697221" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1782245724" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -4080,14 +4307,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778697221" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778697221" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1782245724" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1782245724" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778697221" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1782245724" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -4173,7 +4400,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778697221" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1782245724" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -4184,14 +4411,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778697221" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778697221" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1782245724" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1782245724" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778697221" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1782245724" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -4239,7 +4466,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778697221" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1782245724" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -4250,14 +4477,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778697221" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778697221" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1782245724" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1782245724" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778697221" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1782245724" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -4570,7 +4797,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778697221" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1782245724" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -4581,14 +4808,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778697221" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778697221" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1782245724" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1782245724" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778697221" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1782245724" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -4676,7 +4903,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778697221" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1782245724" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -4687,14 +4914,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778697221" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778697221" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1782245724" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1782245724" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778697221" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1782245724" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -4764,7 +4991,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778697221" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1782245724" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -4775,14 +5002,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778697221" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778697221" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1782245724" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1782245724" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778697221" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1782245724" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -4865,7 +5092,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778697221" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1782245724" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -4876,14 +5103,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778697221" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778697221" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1782245724" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1782245724" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778697221" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1782245724" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -4956,7 +5183,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1778697221" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1782245724" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -4967,14 +5194,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1778697221" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1778697221" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1782245724" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1782245724" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778697221" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1782245724" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>

</xml_diff>

<commit_message>
Got php-zigar working with Zig 0.16.0 (#1052)
</commit_message>
<xml_diff>
--- a/zigar-compiler/test/integration/test-matrix.xlsx
+++ b/zigar-compiler/test/integration/test-matrix.xlsx
@@ -26,17 +26,17 @@
   <calcPr iterateDelta="0.0001"/>
   <extLst>
     <ext uri="smNativeData">
-      <pm:revision xmlns:pm="smNativeData" day="1786163787" val="1234" rev="124" rev64="64" revOS="3" revMin="124" revMax="0"/>
-      <pm:docPrefs xmlns:pm="smNativeData" id="1786163787" fixedDigits="0" showNotice="1" showFrameBounds="1" autoChart="1" recalcOnPrint="1" recalcOnCopy="1" finalRounding="1" compatTextArt="1" tab="567" useDefinedPrintRange="1" printArea="currentSheet"/>
-      <pm:compatibility xmlns:pm="smNativeData" id="1786163787" overlapCells="1"/>
-      <pm:defCurrency xmlns:pm="smNativeData" id="1786163787"/>
+      <pm:revision xmlns:pm="smNativeData" day="1786308497" val="1234" rev="124" rev64="64" revOS="3" revMin="124" revMax="0"/>
+      <pm:docPrefs xmlns:pm="smNativeData" id="1786308497" fixedDigits="0" showNotice="1" showFrameBounds="1" autoChart="1" recalcOnPrint="1" recalcOnCopy="1" finalRounding="1" compatTextArt="1" tab="567" useDefinedPrintRange="1" printArea="currentSheet"/>
+      <pm:compatibility xmlns:pm="smNativeData" id="1786308497" overlapCells="1"/>
+      <pm:defCurrency xmlns:pm="smNativeData" id="1786308497"/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="695" uniqueCount="293">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="811" uniqueCount="293">
   <si>
     <t>Context</t>
   </si>
@@ -116,171 +116,171 @@
     <t>As function parameters</t>
   </si>
   <si>
+    <t>As return value</t>
+  </si>
+  <si>
+    <t>Array of</t>
+  </si>
+  <si>
+    <t>In a struct</t>
+  </si>
+  <si>
+    <t>In a packed struct</t>
+  </si>
+  <si>
+    <t>As comptime field</t>
+  </si>
+  <si>
+    <t>In bare union</t>
+  </si>
+  <si>
+    <t>In tagged union</t>
+  </si>
+  <si>
+    <t>In optional</t>
+  </si>
+  <si>
+    <t>In error union</t>
+  </si>
+  <si>
+    <t>Vector of</t>
+  </si>
+  <si>
+    <t>Scenario</t>
+  </si>
+  <si>
+    <t>Print with newline</t>
+  </si>
+  <si>
+    <t>Print without newline</t>
+  </si>
+  <si>
+    <t>Generate md5 hash</t>
+  </si>
+  <si>
+    <t>Generate sha1 hash</t>
+  </si>
+  <si>
+    <t>Generate CityHash</t>
+  </si>
+  <si>
+    <t>Uncompress gzip data</t>
+  </si>
+  <si>
+    <t>Uncompress xz data</t>
+  </si>
+  <si>
+    <t>Generate random numbers</t>
+  </si>
+  <si>
+    <t>Return total system memory</t>
+  </si>
+  <si>
+    <t>WASM error trace</t>
+  </si>
+  <si>
+    <t>Allow omission of optional struct</t>
+  </si>
+  <si>
+    <t>Throw error</t>
+  </si>
+  <si>
+    <t>Throw error when arguments are off</t>
+  </si>
+  <si>
+    <t>Return slice</t>
+  </si>
+  <si>
+    <t>Return slice of slices</t>
+  </si>
+  <si>
+    <t>Print slice of slices</t>
+  </si>
+  <si>
+    <t>Accept typed array</t>
+  </si>
+  <si>
+    <t>Return bool vector</t>
+  </si>
+  <si>
+    <t>Handle misaligned pointer</t>
+  </si>
+  <si>
+    <t>Handle misaligned aliased pointer</t>
+  </si>
+  <si>
+    <t>Allocate slice of structs</t>
+  </si>
+  <si>
+    <t>Clear pointers</t>
+  </si>
+  <si>
+    <t>Clear pointer array</t>
+  </si>
+  <si>
+    <t>Attach getters/setters</t>
+  </si>
+  <si>
+    <t>Return self-referencing struct</t>
+  </si>
+  <si>
+    <t>Return same struct</t>
+  </si>
+  <si>
+    <t>Allow call as methods</t>
+  </si>
+  <si>
+    <t>Change pointer target</t>
+  </si>
+  <si>
+    <t>Inline function</t>
+  </si>
+  <si>
+    <t>Handle pointers in struct</t>
+  </si>
+  <si>
+    <t>Handle recursive structure</t>
+  </si>
+  <si>
+    <t>Return const pointer</t>
+  </si>
+  <si>
+    <t>Accept multiple pointers</t>
+  </si>
+  <si>
+    <t>Accept C pointers</t>
+  </si>
+  <si>
+    <t>Return C pointers</t>
+  </si>
+  <si>
+    <t>Modify a pointer target</t>
+  </si>
+  <si>
+    <t>Call functions</t>
+  </si>
+  <si>
+    <t>Call variadic functions</t>
+  </si>
+  <si>
+    <t>Pass unsigned in to variadic function</t>
+  </si>
+  <si>
+    <t>Write to file using fwrite</t>
+  </si>
+  <si>
+    <t>Read from file using fread</t>
+  </si>
+  <si>
+    <t>Call printf</t>
+  </si>
+  <si>
+    <t>Call fprintf</t>
+  </si>
+  <si>
     <t>N</t>
   </si>
   <si>
-    <t>As return value</t>
-  </si>
-  <si>
-    <t>Array of</t>
-  </si>
-  <si>
-    <t>In a struct</t>
-  </si>
-  <si>
-    <t>In a packed struct</t>
-  </si>
-  <si>
-    <t>As comptime field</t>
-  </si>
-  <si>
-    <t>In bare union</t>
-  </si>
-  <si>
-    <t>In tagged union</t>
-  </si>
-  <si>
-    <t>In optional</t>
-  </si>
-  <si>
-    <t>In error union</t>
-  </si>
-  <si>
-    <t>Vector of</t>
-  </si>
-  <si>
-    <t>Scenario</t>
-  </si>
-  <si>
-    <t>Print with newline</t>
-  </si>
-  <si>
-    <t>Print without newline</t>
-  </si>
-  <si>
-    <t>Generate md5 hash</t>
-  </si>
-  <si>
-    <t>Generate sha1 hash</t>
-  </si>
-  <si>
-    <t>Generate CityHash</t>
-  </si>
-  <si>
-    <t>Uncompress gzip data</t>
-  </si>
-  <si>
-    <t>Uncompress xz data</t>
-  </si>
-  <si>
-    <t>Generate random numbers</t>
-  </si>
-  <si>
-    <t>Return total system memory</t>
-  </si>
-  <si>
-    <t>WASM error trace</t>
-  </si>
-  <si>
-    <t>Allow omission of optional struct</t>
-  </si>
-  <si>
-    <t>Throw error</t>
-  </si>
-  <si>
-    <t>Throw error when arguments are off</t>
-  </si>
-  <si>
-    <t>Return slice</t>
-  </si>
-  <si>
-    <t>Return slice of slices</t>
-  </si>
-  <si>
-    <t>Print slice of slices</t>
-  </si>
-  <si>
-    <t>Accept typed array</t>
-  </si>
-  <si>
-    <t>Return bool vector</t>
-  </si>
-  <si>
-    <t>Handle misaligned pointer</t>
-  </si>
-  <si>
-    <t>Handle misaligned aliased pointer</t>
-  </si>
-  <si>
-    <t>Allocate slice of structs</t>
-  </si>
-  <si>
-    <t>Clear pointers</t>
-  </si>
-  <si>
-    <t>Clear pointer array</t>
-  </si>
-  <si>
-    <t>Attach getters/setters</t>
-  </si>
-  <si>
-    <t>Return self-referencing struct</t>
-  </si>
-  <si>
-    <t>Return same struct</t>
-  </si>
-  <si>
-    <t>Allow call as methods</t>
-  </si>
-  <si>
-    <t>Change pointer target</t>
-  </si>
-  <si>
-    <t>Inline function</t>
-  </si>
-  <si>
-    <t>Handle pointers in struct</t>
-  </si>
-  <si>
-    <t>Handle recursive structure</t>
-  </si>
-  <si>
-    <t>Return const pointer</t>
-  </si>
-  <si>
-    <t>Accept multiple pointers</t>
-  </si>
-  <si>
-    <t>Accept C pointers</t>
-  </si>
-  <si>
-    <t>Return C pointers</t>
-  </si>
-  <si>
-    <t>Modify a pointer target</t>
-  </si>
-  <si>
-    <t>Call functions</t>
-  </si>
-  <si>
-    <t>Call variadic functions</t>
-  </si>
-  <si>
-    <t>Pass unsigned in to variadic function</t>
-  </si>
-  <si>
-    <t>Write to file using fwrite</t>
-  </si>
-  <si>
-    <t>Read from file using fread</t>
-  </si>
-  <si>
-    <t>Call printf</t>
-  </si>
-  <si>
-    <t>Call fprintf</t>
-  </si>
-  <si>
     <t>Call sprintf</t>
   </si>
   <si>
@@ -536,7 +536,7 @@
     <t>Open and read file in main thread</t>
   </si>
   <si>
-    <t>Fall to to system</t>
+    <t>Fall thru to system</t>
   </si>
   <si>
     <t>Open file through FS using posix functions</t>
@@ -944,7 +944,7 @@
       <sz val="11"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1786163787" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1786308497" ulstyle="none" kern="1">
             <pm:latin face="Calibri" sz="220" lang="default"/>
             <pm:cs face="Basic Roman" sz="220" lang="default"/>
             <pm:ea face="Basic Roman" sz="220" lang="default"/>
@@ -959,7 +959,7 @@
       <sz val="10"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1786163787" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1786308497" ulstyle="none" kern="1">
             <pm:latin face="Basic Sans" sz="200" lang="default"/>
             <pm:cs face="Basic Roman" sz="200" lang="default"/>
             <pm:ea face="Basic Roman" sz="200" lang="default"/>
@@ -974,7 +974,7 @@
       <sz val="10"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1786163787" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1786308497" ulstyle="none" kern="1">
             <pm:latin face="Arial" sz="200" lang="default"/>
             <pm:cs face="Basic Roman" sz="200" lang="default"/>
             <pm:ea face="Basic Roman" sz="200" lang="default"/>
@@ -990,7 +990,7 @@
       <sz val="11"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1786163787" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1786308497" ulstyle="none" kern="1">
             <pm:latin face="Calibri" sz="220" lang="default" weight="bold"/>
             <pm:cs face="Basic Roman" sz="220" lang="default" weight="bold"/>
             <pm:ea face="Basic Roman" sz="220" lang="default" weight="bold"/>
@@ -999,7 +999,7 @@
       </extLst>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1012,7 +1012,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1786163787" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
+            <pm:shade xmlns:pm="smNativeData" id="1786308497" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
           </ext>
         </extLst>
       </patternFill>
@@ -1023,7 +1023,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1786163787" type="1" fgLvl="100" fgClr="0081D41A" bgLvl="0" bgClr="0092D050"/>
+            <pm:shade xmlns:pm="smNativeData" id="1786308497" type="1" fgLvl="100" fgClr="0081D41A" bgLvl="0" bgClr="0092D050"/>
           </ext>
         </extLst>
       </patternFill>
@@ -1034,7 +1034,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1786163787" type="1" fgLvl="100" fgClr="0092D050" bgLvl="0" bgClr="0081D41A"/>
+            <pm:shade xmlns:pm="smNativeData" id="1786308497" type="1" fgLvl="100" fgClr="0092D050" bgLvl="0" bgClr="0081D41A"/>
           </ext>
         </extLst>
       </patternFill>
@@ -1045,7 +1045,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1786163787" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
+            <pm:shade xmlns:pm="smNativeData" id="1786308497" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
           </ext>
         </extLst>
       </patternFill>
@@ -1056,7 +1056,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1786163787" type="1" fgLvl="100" fgClr="00999999" bgLvl="0" bgClr="00808080"/>
+            <pm:shade xmlns:pm="smNativeData" id="1786308497" type="1" fgLvl="100" fgClr="00999999" bgLvl="0" bgClr="00808080"/>
           </ext>
         </extLst>
       </patternFill>
@@ -1067,7 +1067,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1786163787" type="1" fgLvl="100" fgClr="00FFFFFF" bgLvl="100" bgClr="00000000"/>
+            <pm:shade xmlns:pm="smNativeData" id="1786308497" type="1" fgLvl="100" fgClr="00FFFFFF" bgLvl="100" bgClr="00000000"/>
           </ext>
         </extLst>
       </patternFill>
@@ -1078,13 +1078,24 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1786163787" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
+            <pm:shade xmlns:pm="smNativeData" id="1786308497" type="1" fgLvl="100" fgClr="00FFC000" bgLvl="0" bgClr="00FF9900"/>
+          </ext>
+        </extLst>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFB3B3"/>
+        <bgColor rgb="FFFFFFFF"/>
+        <extLst>
+          <ext uri="smNativeData">
+            <pm:shade xmlns:pm="smNativeData" id="1786308497" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="100" bgClr="00FFFFFF"/>
           </ext>
         </extLst>
       </patternFill>
     </fill>
   </fills>
-  <borders count="8">
+  <borders count="9">
     <border>
       <left style="none">
         <color rgb="FF000000"/>
@@ -1100,7 +1111,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1786163787"/>
+          <pm:border xmlns:pm="smNativeData" id="1786308497"/>
         </ext>
       </extLst>
     </border>
@@ -1119,7 +1130,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1786163787">
+          <pm:border xmlns:pm="smNativeData" id="1786308497">
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="right" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
           </pm:border>
@@ -1141,7 +1152,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1786163787">
+          <pm:border xmlns:pm="smNativeData" id="1786308497">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -1165,7 +1176,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1786163787">
+          <pm:border xmlns:pm="smNativeData" id="1786308497">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -1189,7 +1200,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1786163787">
+          <pm:border xmlns:pm="smNativeData" id="1786308497">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -1213,7 +1224,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1786163787"/>
+          <pm:border xmlns:pm="smNativeData" id="1786308497"/>
         </ext>
       </extLst>
     </border>
@@ -1232,7 +1243,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1786163787"/>
+          <pm:border xmlns:pm="smNativeData" id="1786308497"/>
         </ext>
       </extLst>
     </border>
@@ -1251,7 +1262,26 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1786163787"/>
+          <pm:border xmlns:pm="smNativeData" id="1786308497"/>
+        </ext>
+      </extLst>
+    </border>
+    <border>
+      <left style="none">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="none">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="none">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="none">
+        <color rgb="FF000000"/>
+      </bottom>
+      <extLst>
+        <ext uri="smNativeData">
+          <pm:border xmlns:pm="smNativeData" id="1786308497"/>
         </ext>
       </extLst>
     </border>
@@ -1304,7 +1334,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1786163787" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1786308497" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1317,7 +1347,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1786163787" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1786308497" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1328,7 +1358,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1786163787" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1786308497" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1341,7 +1371,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1786163787" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1786308497" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1352,7 +1382,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1786163787" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1786308497" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1365,7 +1395,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1786163787" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1786308497" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1376,7 +1406,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1786163787" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1786308497" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1389,7 +1419,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1786163787" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1786308497" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1400,7 +1430,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1786163787" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1786308497" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1413,7 +1443,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1786163787" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1786308497" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1424,7 +1454,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1786163787" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1786308497" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1437,7 +1467,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1786163787" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1786308497" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1448,7 +1478,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1786163787" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1786308497" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1461,7 +1491,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1786163787" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1786308497" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1472,7 +1502,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1786163787" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1786308497" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1485,7 +1515,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1786163787" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1786308497" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1496,7 +1526,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1786163787" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1786308497" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1509,7 +1539,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1786163787" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1786308497" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1520,7 +1550,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1786163787" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1786308497" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1533,7 +1563,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1786163787" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1786308497" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1544,7 +1574,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1786163787" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1786308497" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1557,7 +1587,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1786163787" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1786308497" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1568,7 +1598,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1786163787" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1786308497" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1581,7 +1611,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1786163787" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1786308497" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1592,7 +1622,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1786163787" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1786308497" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1605,7 +1635,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1786163787" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1786308497" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1616,7 +1646,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1786163787" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1786308497" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1629,7 +1659,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1786163787" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1786308497" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1640,7 +1670,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1786163787" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1786308497" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1653,7 +1683,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1786163787" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1786308497" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1664,7 +1694,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1786163787" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1786308497" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1677,7 +1707,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1786163787" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1786308497" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1688,7 +1718,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1786163787" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1786308497" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1701,7 +1731,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1786163787" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1786308497" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1712,7 +1742,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1786163787" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1786308497" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1725,7 +1755,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1786163787" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1786308497" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1736,7 +1766,7 @@
         <color rgb="FFFF0000"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:charSpec xmlns:pm="smNativeData" id="1786163787" fgClr="FF0000">
+            <pm:charSpec xmlns:pm="smNativeData" id="1786308497" fgClr="FF0000">
               <pm:latin/>
               <pm:cs/>
               <pm:ea/>
@@ -1749,7 +1779,7 @@
           <bgColor rgb="FFFFB3B3"/>
           <extLst>
             <ext uri="smNativeData">
-              <pm:shade xmlns:pm="smNativeData" id="1786163787" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
+              <pm:shade xmlns:pm="smNativeData" id="1786308497" type="1" fgLvl="30" fgClr="00FF0000" bgLvl="255" bgClr="00FFFFFF"/>
             </ext>
           </extLst>
         </patternFill>
@@ -1759,10 +1789,10 @@
   <tableStyles count="0"/>
   <extLst>
     <ext uri="smNativeData">
-      <pm:charStyles xmlns:pm="smNativeData" id="1786163787" count="1">
+      <pm:charStyles xmlns:pm="smNativeData" id="1786308497" count="1">
         <pm:charStyle name="Normal" fontId="0" Id="1"/>
       </pm:charStyles>
-      <pm:colors xmlns:pm="smNativeData" id="1786163787" count="6">
+      <pm:colors xmlns:pm="smNativeData" id="1786308497" count="6">
         <pm:color name="Color 24" rgb="FFC000"/>
         <pm:color name="Color 25" rgb="FF9900"/>
         <pm:color name="Color 26" rgb="81D41A"/>
@@ -2287,7 +2317,7 @@
         <v>24</v>
       </c>
       <c r="T4" s="10" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="U4" s="10" t="s">
         <v>24</v>
@@ -2301,7 +2331,7 @@
     </row>
     <row r="5" spans="1:23">
       <c r="A5" s="9" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B5" s="10" t="s">
         <v>24</v>
@@ -2372,7 +2402,7 @@
     </row>
     <row r="6" spans="1:23">
       <c r="A6" s="9" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B6" s="10" t="s">
         <v>24</v>
@@ -2443,7 +2473,7 @@
     </row>
     <row r="7" spans="1:23">
       <c r="A7" s="9" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B7" s="10" t="s">
         <v>24</v>
@@ -2514,7 +2544,7 @@
     </row>
     <row r="8" spans="1:23">
       <c r="A8" s="9" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B8" s="10" t="s">
         <v>24</v>
@@ -2535,7 +2565,7 @@
         <v>24</v>
       </c>
       <c r="H8" s="10" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="I8" s="10" t="s">
         <v>24</v>
@@ -2574,10 +2604,10 @@
         <v>24</v>
       </c>
       <c r="U8" s="10" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="V8" s="10" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="W8" s="10" t="s">
         <v>24</v>
@@ -2585,7 +2615,7 @@
     </row>
     <row r="9" spans="1:23">
       <c r="A9" s="9" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B9" s="10" t="s">
         <v>24</v>
@@ -2656,7 +2686,7 @@
     </row>
     <row r="10" spans="1:23">
       <c r="A10" s="9" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B10" s="10" t="s">
         <v>24</v>
@@ -2727,7 +2757,7 @@
     </row>
     <row r="11" spans="1:23">
       <c r="A11" s="9" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B11" s="10" t="s">
         <v>24</v>
@@ -2798,7 +2828,7 @@
     </row>
     <row r="12" spans="1:23">
       <c r="A12" s="9" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B12" s="10" t="s">
         <v>24</v>
@@ -2869,7 +2899,7 @@
     </row>
     <row r="13" spans="1:23">
       <c r="A13" s="9" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B13" s="10" t="s">
         <v>24</v>
@@ -2940,7 +2970,7 @@
     </row>
     <row r="14" spans="1:23">
       <c r="A14" s="9" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B14" s="10" t="s">
         <v>24</v>
@@ -3032,7 +3062,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1786163787" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1786308497" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3041,14 +3071,14 @@
   <headerFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1786163787" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1786163787" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1786308497" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1786308497" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1786163787" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1786308497" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3067,7 +3097,7 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B1" s="11"/>
     </row>
@@ -3128,7 +3158,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1786163787" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1786308497" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3139,14 +3169,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1786163787" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1786163787" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1786308497" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1786308497" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1786163787" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1786308497" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3166,7 +3196,7 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B1" s="11"/>
     </row>
@@ -3211,7 +3241,7 @@
         <v>159</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -3219,7 +3249,7 @@
         <v>160</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="9" spans="1:2">
@@ -3227,7 +3257,7 @@
         <v>161</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="10" spans="1:2">
@@ -3235,7 +3265,7 @@
         <v>162</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
   </sheetData>
@@ -3256,7 +3286,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1786163787" printRowHead="0" printColHead="0" printHeadLine="0" printFootLine="0" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1786308497" printRowHead="0" printColHead="0" printHeadLine="0" printFootLine="0" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3265,14 +3295,14 @@
   <headerFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1786163787" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1786163787" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1786308497" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1786308497" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1786163787" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1786308497" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3292,7 +3322,7 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B1" s="11"/>
     </row>
@@ -3304,710 +3334,946 @@
       <c r="A3" s="9" t="s">
         <v>163</v>
       </c>
-      <c r="B3" s="10"/>
+      <c r="B3" s="10" t="s">
+        <v>24</v>
+      </c>
       <c r="D3" s="10"/>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
         <v>164</v>
       </c>
-      <c r="B4" s="10"/>
+      <c r="B4" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
         <v>165</v>
       </c>
-      <c r="B5" s="10"/>
+      <c r="B5" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="9" t="s">
         <v>166</v>
       </c>
-      <c r="B6" s="10"/>
+      <c r="B6" s="10" t="s">
+        <v>80</v>
+      </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="9" t="s">
         <v>167</v>
       </c>
-      <c r="B7" s="10"/>
+      <c r="B7" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="9" t="s">
         <v>168</v>
       </c>
-      <c r="B8" s="10"/>
+      <c r="B8" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="9" t="s">
         <v>169</v>
       </c>
-      <c r="B9" s="10"/>
+      <c r="B9" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="9" t="s">
         <v>170</v>
       </c>
-      <c r="B10" s="10"/>
+      <c r="B10" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="9" t="s">
         <v>171</v>
       </c>
-      <c r="B11" s="10"/>
+      <c r="B11" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="9" t="s">
         <v>172</v>
       </c>
-      <c r="B12" s="10"/>
+      <c r="B12" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="9" t="s">
         <v>173</v>
       </c>
-      <c r="B13" s="10"/>
+      <c r="B13" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="9" t="s">
         <v>174</v>
       </c>
-      <c r="B14" s="10"/>
+      <c r="B14" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="15" spans="1:2">
       <c r="A15" s="9" t="s">
         <v>175</v>
       </c>
-      <c r="B15" s="10"/>
+      <c r="B15" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="16" spans="1:2">
       <c r="A16" s="9" t="s">
         <v>176</v>
       </c>
-      <c r="B16" s="10"/>
+      <c r="B16" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="9" t="s">
         <v>177</v>
       </c>
-      <c r="B17" s="10"/>
+      <c r="B17" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="18" spans="1:2">
       <c r="A18" s="9" t="s">
         <v>178</v>
       </c>
-      <c r="B18" s="10"/>
+      <c r="B18" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="19" spans="1:2">
       <c r="A19" s="9" t="s">
         <v>179</v>
       </c>
-      <c r="B19" s="10"/>
+      <c r="B19" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="20" spans="1:2">
       <c r="A20" s="9" t="s">
         <v>180</v>
       </c>
-      <c r="B20" s="10"/>
+      <c r="B20" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="21" spans="1:2">
       <c r="A21" s="9" t="s">
         <v>181</v>
       </c>
-      <c r="B21" s="10"/>
+      <c r="B21" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="22" spans="1:2">
       <c r="A22" s="9" t="s">
         <v>182</v>
       </c>
-      <c r="B22" s="10"/>
+      <c r="B22" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="23" spans="1:2">
       <c r="A23" s="9" t="s">
         <v>183</v>
       </c>
-      <c r="B23" s="10"/>
+      <c r="B23" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="24" spans="1:2">
       <c r="A24" s="9" t="s">
         <v>184</v>
       </c>
-      <c r="B24" s="10"/>
+      <c r="B24" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="25" spans="1:2">
       <c r="A25" s="9" t="s">
         <v>185</v>
       </c>
-      <c r="B25" s="10"/>
+      <c r="B25" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="26" spans="1:2">
       <c r="A26" s="9" t="s">
         <v>186</v>
       </c>
-      <c r="B26" s="10"/>
+      <c r="B26" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="27" spans="1:2">
       <c r="A27" s="9" t="s">
         <v>187</v>
       </c>
-      <c r="B27" s="10"/>
+      <c r="B27" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="28" spans="1:2">
       <c r="A28" s="9" t="s">
         <v>188</v>
       </c>
-      <c r="B28" s="10"/>
+      <c r="B28" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="29" spans="1:2">
       <c r="A29" s="9" t="s">
         <v>189</v>
       </c>
-      <c r="B29" s="10"/>
+      <c r="B29" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="30" spans="1:2">
       <c r="A30" s="9" t="s">
         <v>190</v>
       </c>
-      <c r="B30" s="10"/>
+      <c r="B30" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="31" spans="1:2">
       <c r="A31" s="9" t="s">
         <v>191</v>
       </c>
-      <c r="B31" s="10"/>
+      <c r="B31" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="32" spans="1:2">
       <c r="A32" s="9" t="s">
         <v>192</v>
       </c>
-      <c r="B32" s="10"/>
+      <c r="B32" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="33" spans="1:2">
       <c r="A33" s="9" t="s">
         <v>193</v>
       </c>
-      <c r="B33" s="10"/>
+      <c r="B33" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="34" spans="1:2">
       <c r="A34" s="9" t="s">
         <v>194</v>
       </c>
-      <c r="B34" s="10"/>
+      <c r="B34" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="35" spans="1:2">
       <c r="A35" s="9" t="s">
         <v>195</v>
       </c>
-      <c r="B35" s="10"/>
+      <c r="B35" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="36" spans="1:2">
       <c r="A36" s="9" t="s">
         <v>196</v>
       </c>
-      <c r="B36" s="10"/>
+      <c r="B36" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="37" spans="1:2">
       <c r="A37" s="9" t="s">
         <v>197</v>
       </c>
-      <c r="B37" s="10"/>
+      <c r="B37" s="10" t="s">
+        <v>80</v>
+      </c>
     </row>
     <row r="38" spans="1:2">
       <c r="A38" s="9" t="s">
         <v>198</v>
       </c>
-      <c r="B38" s="10"/>
+      <c r="B38" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="39" spans="1:2">
       <c r="A39" s="9" t="s">
         <v>199</v>
       </c>
-      <c r="B39" s="10"/>
+      <c r="B39" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="40" spans="1:2">
       <c r="A40" s="9" t="s">
         <v>200</v>
       </c>
-      <c r="B40" s="10"/>
+      <c r="B40" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="41" spans="1:2">
       <c r="A41" s="9" t="s">
         <v>201</v>
       </c>
-      <c r="B41" s="10"/>
+      <c r="B41" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="42" spans="1:2">
       <c r="A42" s="9" t="s">
         <v>202</v>
       </c>
-      <c r="B42" s="10"/>
+      <c r="B42" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="43" spans="1:2">
       <c r="A43" s="9" t="s">
         <v>203</v>
       </c>
-      <c r="B43" s="10"/>
+      <c r="B43" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="44" spans="1:2">
       <c r="A44" s="9" t="s">
         <v>204</v>
       </c>
-      <c r="B44" s="10"/>
+      <c r="B44" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="45" spans="1:2">
       <c r="A45" s="9" t="s">
         <v>205</v>
       </c>
-      <c r="B45" s="10"/>
+      <c r="B45" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="46" spans="1:2">
       <c r="A46" s="9" t="s">
         <v>206</v>
       </c>
-      <c r="B46" s="10"/>
+      <c r="B46" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="47" spans="1:2">
       <c r="A47" s="9" t="s">
         <v>207</v>
       </c>
-      <c r="B47" s="10"/>
+      <c r="B47" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="48" spans="1:2">
       <c r="A48" s="9" t="s">
         <v>208</v>
       </c>
-      <c r="B48" s="10"/>
+      <c r="B48" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="49" spans="1:2">
       <c r="A49" s="9" t="s">
         <v>209</v>
       </c>
-      <c r="B49" s="10"/>
+      <c r="B49" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="50" spans="1:2">
       <c r="A50" s="9" t="s">
         <v>210</v>
       </c>
-      <c r="B50" s="10"/>
+      <c r="B50" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="51" spans="1:2">
       <c r="A51" s="9" t="s">
         <v>211</v>
       </c>
-      <c r="B51" s="10"/>
+      <c r="B51" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="52" spans="1:2">
       <c r="A52" s="9" t="s">
         <v>212</v>
       </c>
-      <c r="B52" s="10"/>
+      <c r="B52" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="53" spans="1:2">
       <c r="A53" s="9" t="s">
         <v>213</v>
       </c>
-      <c r="B53" s="10"/>
+      <c r="B53" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="54" spans="1:2">
       <c r="A54" s="9" t="s">
         <v>214</v>
       </c>
-      <c r="B54" s="10"/>
+      <c r="B54" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="55" spans="1:2">
       <c r="A55" s="9" t="s">
         <v>215</v>
       </c>
-      <c r="B55" s="10"/>
+      <c r="B55" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="56" spans="1:2">
       <c r="A56" s="9" t="s">
         <v>216</v>
       </c>
-      <c r="B56" s="10"/>
+      <c r="B56" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="57" spans="1:2">
       <c r="A57" s="9" t="s">
         <v>217</v>
       </c>
-      <c r="B57" s="10"/>
+      <c r="B57" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="58" spans="1:2">
       <c r="A58" s="9" t="s">
         <v>218</v>
       </c>
-      <c r="B58" s="10"/>
+      <c r="B58" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="59" spans="1:2">
       <c r="A59" s="9" t="s">
         <v>219</v>
       </c>
-      <c r="B59" s="10"/>
+      <c r="B59" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="60" spans="1:2">
       <c r="A60" s="9" t="s">
         <v>220</v>
       </c>
-      <c r="B60" s="10"/>
+      <c r="B60" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="61" spans="1:2">
       <c r="A61" s="9" t="s">
         <v>221</v>
       </c>
-      <c r="B61" s="10"/>
+      <c r="B61" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="62" spans="1:2">
       <c r="A62" s="9" t="s">
         <v>222</v>
       </c>
-      <c r="B62" s="10"/>
+      <c r="B62" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="63" spans="1:2">
       <c r="A63" s="9" t="s">
         <v>223</v>
       </c>
-      <c r="B63" s="10"/>
+      <c r="B63" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="64" spans="1:2">
       <c r="A64" s="9" t="s">
         <v>224</v>
       </c>
-      <c r="B64" s="10"/>
+      <c r="B64" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="65" spans="1:2">
       <c r="A65" s="9" t="s">
         <v>225</v>
       </c>
-      <c r="B65" s="10"/>
+      <c r="B65" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="66" spans="1:2">
       <c r="A66" s="9" t="s">
         <v>226</v>
       </c>
-      <c r="B66" s="10"/>
+      <c r="B66" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="67" spans="1:2">
       <c r="A67" s="9" t="s">
         <v>227</v>
       </c>
-      <c r="B67" s="10"/>
+      <c r="B67" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="68" spans="1:2">
       <c r="A68" s="9" t="s">
         <v>228</v>
       </c>
-      <c r="B68" s="10"/>
+      <c r="B68" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="69" spans="1:2">
       <c r="A69" s="9" t="s">
         <v>229</v>
       </c>
-      <c r="B69" s="10"/>
+      <c r="B69" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="70" spans="1:2">
       <c r="A70" s="9" t="s">
         <v>230</v>
       </c>
-      <c r="B70" s="10"/>
+      <c r="B70" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="71" spans="1:2">
       <c r="A71" s="9" t="s">
         <v>231</v>
       </c>
-      <c r="B71" s="10"/>
+      <c r="B71" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="72" spans="1:2">
       <c r="A72" s="9" t="s">
         <v>232</v>
       </c>
-      <c r="B72" s="10"/>
+      <c r="B72" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="73" spans="1:2">
       <c r="A73" s="9" t="s">
         <v>233</v>
       </c>
-      <c r="B73" s="10"/>
+      <c r="B73" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="74" spans="1:2">
       <c r="A74" s="9" t="s">
         <v>234</v>
       </c>
-      <c r="B74" s="10"/>
+      <c r="B74" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="75" spans="1:2">
       <c r="A75" s="9" t="s">
         <v>235</v>
       </c>
-      <c r="B75" s="10"/>
+      <c r="B75" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="76" spans="1:2">
       <c r="A76" s="9" t="s">
         <v>236</v>
       </c>
-      <c r="B76" s="10"/>
+      <c r="B76" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="77" spans="1:2">
       <c r="A77" s="9" t="s">
         <v>237</v>
       </c>
-      <c r="B77" s="10"/>
+      <c r="B77" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="78" spans="1:2">
       <c r="A78" s="9" t="s">
         <v>238</v>
       </c>
-      <c r="B78" s="10"/>
+      <c r="B78" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="79" spans="1:2">
       <c r="A79" s="9" t="s">
         <v>239</v>
       </c>
-      <c r="B79" s="10"/>
+      <c r="B79" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="80" spans="1:2">
       <c r="A80" s="9" t="s">
         <v>240</v>
       </c>
-      <c r="B80" s="10"/>
+      <c r="B80" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="81" spans="1:2">
       <c r="A81" s="9" t="s">
         <v>241</v>
       </c>
-      <c r="B81" s="10"/>
+      <c r="B81" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="82" spans="1:2">
       <c r="A82" s="9" t="s">
         <v>242</v>
       </c>
-      <c r="B82" s="10"/>
+      <c r="B82" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="83" spans="1:2">
       <c r="A83" s="9" t="s">
         <v>243</v>
       </c>
-      <c r="B83" s="10"/>
+      <c r="B83" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="84" spans="1:2">
       <c r="A84" s="9" t="s">
         <v>244</v>
       </c>
-      <c r="B84" s="10"/>
+      <c r="B84" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="85" spans="1:2">
       <c r="A85" s="9" t="s">
         <v>245</v>
       </c>
-      <c r="B85" s="10"/>
+      <c r="B85" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="86" spans="1:2">
       <c r="A86" s="9" t="s">
         <v>246</v>
       </c>
-      <c r="B86" s="10"/>
+      <c r="B86" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="87" spans="1:2">
       <c r="A87" s="9" t="s">
         <v>247</v>
       </c>
-      <c r="B87" s="10"/>
+      <c r="B87" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="88" spans="1:2">
       <c r="A88" s="9" t="s">
         <v>248</v>
       </c>
-      <c r="B88" s="10"/>
+      <c r="B88" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="89" spans="1:2">
       <c r="A89" s="9" t="s">
         <v>249</v>
       </c>
-      <c r="B89" s="10"/>
+      <c r="B89" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="90" spans="1:2">
       <c r="A90" s="9" t="s">
         <v>250</v>
       </c>
-      <c r="B90" s="10"/>
+      <c r="B90" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="91" spans="1:2">
       <c r="A91" s="9" t="s">
         <v>251</v>
       </c>
-      <c r="B91" s="10"/>
+      <c r="B91" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="92" spans="1:2">
       <c r="A92" s="9" t="s">
         <v>252</v>
       </c>
-      <c r="B92" s="10"/>
+      <c r="B92" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="93" spans="1:2">
       <c r="A93" s="9" t="s">
         <v>253</v>
       </c>
-      <c r="B93" s="10"/>
+      <c r="B93" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="94" spans="1:2">
       <c r="A94" s="9" t="s">
         <v>254</v>
       </c>
-      <c r="B94" s="10"/>
+      <c r="B94" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="95" spans="1:2">
       <c r="A95" s="9" t="s">
         <v>255</v>
       </c>
-      <c r="B95" s="10"/>
+      <c r="B95" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="96" spans="1:2">
       <c r="A96" s="9" t="s">
         <v>256</v>
       </c>
-      <c r="B96" s="10"/>
+      <c r="B96" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="97" spans="1:2">
       <c r="A97" s="9" t="s">
         <v>257</v>
       </c>
-      <c r="B97" s="10"/>
+      <c r="B97" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="98" spans="1:2">
       <c r="A98" s="9" t="s">
         <v>258</v>
       </c>
-      <c r="B98" s="10"/>
+      <c r="B98" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="99" spans="1:2">
       <c r="A99" s="9" t="s">
         <v>259</v>
       </c>
-      <c r="B99" s="10"/>
+      <c r="B99" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="100" spans="1:2">
       <c r="A100" s="9" t="s">
         <v>260</v>
       </c>
-      <c r="B100" s="10"/>
+      <c r="B100" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="101" spans="1:2">
       <c r="A101" s="9" t="s">
         <v>261</v>
       </c>
-      <c r="B101" s="10"/>
+      <c r="B101" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="102" spans="1:2">
       <c r="A102" s="9" t="s">
         <v>262</v>
       </c>
-      <c r="B102" s="10"/>
+      <c r="B102" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="103" spans="1:2">
       <c r="A103" s="9" t="s">
         <v>263</v>
       </c>
-      <c r="B103" s="10"/>
+      <c r="B103" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="104" spans="1:2">
       <c r="A104" s="9" t="s">
         <v>264</v>
       </c>
-      <c r="B104" s="10"/>
+      <c r="B104" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="105" spans="1:2">
       <c r="A105" s="9" t="s">
         <v>265</v>
       </c>
-      <c r="B105" s="10"/>
+      <c r="B105" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="106" spans="1:2">
       <c r="A106" s="9" t="s">
         <v>266</v>
       </c>
-      <c r="B106" s="10"/>
+      <c r="B106" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="107" spans="1:2">
       <c r="A107" s="9" t="s">
         <v>267</v>
       </c>
-      <c r="B107" s="10"/>
+      <c r="B107" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="108" spans="1:2">
       <c r="A108" s="9" t="s">
         <v>268</v>
       </c>
-      <c r="B108" s="10"/>
+      <c r="B108" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="109" spans="1:2">
       <c r="A109" s="9" t="s">
         <v>269</v>
       </c>
-      <c r="B109" s="10"/>
+      <c r="B109" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="110" spans="1:2">
       <c r="A110" s="9" t="s">
         <v>270</v>
       </c>
-      <c r="B110" s="10"/>
+      <c r="B110" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="111" spans="1:2">
       <c r="A111" s="9" t="s">
         <v>271</v>
       </c>
-      <c r="B111" s="10"/>
+      <c r="B111" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="112" spans="1:2">
       <c r="A112" s="9" t="s">
         <v>272</v>
       </c>
-      <c r="B112" s="10"/>
+      <c r="B112" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="113" spans="1:2">
       <c r="A113" s="9" t="s">
         <v>273</v>
       </c>
-      <c r="B113" s="10"/>
+      <c r="B113" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="114" spans="1:2">
       <c r="A114" s="9" t="s">
         <v>274</v>
       </c>
-      <c r="B114" s="10"/>
+      <c r="B114" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="115" spans="1:2">
       <c r="A115" s="9" t="s">
         <v>275</v>
       </c>
-      <c r="B115" s="10"/>
+      <c r="B115" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="116" spans="1:2">
       <c r="A116" s="9" t="s">
         <v>276</v>
       </c>
-      <c r="B116" s="10"/>
+      <c r="B116" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="117" spans="1:2">
       <c r="A117" s="9" t="s">
         <v>277</v>
       </c>
-      <c r="B117" s="10"/>
+      <c r="B117" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="118" spans="1:2">
       <c r="A118" s="9" t="s">
         <v>278</v>
       </c>
-      <c r="B118" s="10"/>
+      <c r="B118" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="119" spans="1:2">
       <c r="A119" s="9" t="s">
         <v>279</v>
       </c>
-      <c r="B119" s="10"/>
+      <c r="B119" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="120" spans="1:2">
       <c r="A120" s="9" t="s">
         <v>280</v>
       </c>
-      <c r="B120" s="10"/>
+      <c r="B120" s="10" t="s">
+        <v>24</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -4022,7 +4288,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1786163787" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1786308497" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -4033,14 +4299,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1786163787" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1786163787" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1786308497" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1786308497" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1786163787" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1786308497" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -4059,7 +4325,7 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B1" s="11"/>
     </row>
@@ -4152,7 +4418,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1786163787" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1786308497" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -4163,14 +4429,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1786163787" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1786163787" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1786308497" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1786308497" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1786163787" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1786308497" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -4189,7 +4455,7 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B1" s="11"/>
     </row>
@@ -4218,7 +4484,7 @@
         <v>292</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
   </sheetData>
@@ -4234,7 +4500,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1786163787" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1786308497" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -4245,14 +4511,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1786163787" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1786163787" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1786308497" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1786308497" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1786163787" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1786308497" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -4271,7 +4537,7 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B1" s="11"/>
     </row>
@@ -4281,7 +4547,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B3" s="10" t="s">
         <v>24</v>
@@ -4289,7 +4555,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B4" s="10" t="s">
         <v>24</v>
@@ -4308,7 +4574,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1786163787" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1786308497" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -4319,14 +4585,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1786163787" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1786163787" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1786308497" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1786308497" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1786163787" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1786308497" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -4345,7 +4611,7 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B1" s="11"/>
     </row>
@@ -4355,7 +4621,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B3" s="10" t="s">
         <v>24</v>
@@ -4363,7 +4629,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B4" s="10" t="s">
         <v>24</v>
@@ -4371,31 +4637,31 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B5" s="10"/>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="9" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B6" s="10"/>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="9" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B7" s="10"/>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="9" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B8" s="10"/>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="9" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B9" s="10"/>
     </row>
@@ -4412,7 +4678,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1786163787" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1786308497" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -4423,14 +4689,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1786163787" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1786163787" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1786308497" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1786308497" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1786163787" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1786308497" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -4449,7 +4715,7 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B1" s="11"/>
     </row>
@@ -4459,7 +4725,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B3" s="10"/>
     </row>
@@ -4476,7 +4742,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1786163787" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1786308497" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -4487,14 +4753,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1786163787" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1786163787" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1786308497" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1786308497" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1786163787" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1786308497" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -4513,7 +4779,7 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B1" s="11"/>
     </row>
@@ -4523,7 +4789,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B3" s="10" t="s">
         <v>24</v>
@@ -4531,7 +4797,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B4" s="10" t="s">
         <v>24</v>
@@ -4539,7 +4805,7 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B5" s="10" t="s">
         <v>24</v>
@@ -4547,7 +4813,7 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="9" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B6" s="10" t="s">
         <v>24</v>
@@ -4555,7 +4821,7 @@
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="9" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B7" s="10" t="s">
         <v>24</v>
@@ -4563,7 +4829,7 @@
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="9" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B8" s="10" t="s">
         <v>24</v>
@@ -4571,7 +4837,7 @@
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="9" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B9" s="10" t="s">
         <v>24</v>
@@ -4579,7 +4845,7 @@
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="9" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B10" s="10" t="s">
         <v>24</v>
@@ -4587,7 +4853,7 @@
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="9" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B11" s="10" t="s">
         <v>24</v>
@@ -4595,7 +4861,7 @@
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="9" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B12" s="10" t="s">
         <v>24</v>
@@ -4603,7 +4869,7 @@
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="9" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B13" s="10" t="s">
         <v>24</v>
@@ -4611,7 +4877,7 @@
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="9" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B14" s="10" t="s">
         <v>24</v>
@@ -4619,7 +4885,7 @@
     </row>
     <row r="15" spans="1:2">
       <c r="A15" s="9" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B15" s="10" t="s">
         <v>24</v>
@@ -4627,7 +4893,7 @@
     </row>
     <row r="16" spans="1:2">
       <c r="A16" s="9" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B16" s="10" t="s">
         <v>24</v>
@@ -4635,7 +4901,7 @@
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="9" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B17" s="10" t="s">
         <v>24</v>
@@ -4643,7 +4909,7 @@
     </row>
     <row r="18" spans="1:2">
       <c r="A18" s="9" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B18" s="10" t="s">
         <v>24</v>
@@ -4651,7 +4917,7 @@
     </row>
     <row r="19" spans="1:2">
       <c r="A19" s="9" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B19" s="10" t="s">
         <v>24</v>
@@ -4659,7 +4925,7 @@
     </row>
     <row r="20" spans="1:2">
       <c r="A20" s="9" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B20" s="10" t="s">
         <v>24</v>
@@ -4667,7 +4933,7 @@
     </row>
     <row r="21" spans="1:2">
       <c r="A21" s="9" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B21" s="10" t="s">
         <v>24</v>
@@ -4675,7 +4941,7 @@
     </row>
     <row r="22" spans="1:2">
       <c r="A22" s="9" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B22" s="10" t="s">
         <v>24</v>
@@ -4683,7 +4949,7 @@
     </row>
     <row r="23" spans="1:2">
       <c r="A23" s="9" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B23" s="10" t="s">
         <v>24</v>
@@ -4691,7 +4957,7 @@
     </row>
     <row r="24" spans="1:2">
       <c r="A24" s="9" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B24" s="10" t="s">
         <v>24</v>
@@ -4699,7 +4965,7 @@
     </row>
     <row r="25" spans="1:4">
       <c r="A25" s="9" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B25" s="10" t="s">
         <v>24</v>
@@ -4708,7 +4974,7 @@
     </row>
     <row r="26" spans="1:4">
       <c r="A26" s="9" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B26" s="10" t="s">
         <v>24</v>
@@ -4717,7 +4983,7 @@
     </row>
     <row r="27" spans="1:4">
       <c r="A27" s="9" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B27" s="10" t="s">
         <v>24</v>
@@ -4726,7 +4992,7 @@
     </row>
     <row r="28" spans="1:4">
       <c r="A28" s="9" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B28" s="10" t="s">
         <v>24</v>
@@ -4735,7 +5001,7 @@
     </row>
     <row r="29" spans="1:4">
       <c r="A29" s="9" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B29" s="10" t="s">
         <v>24</v>
@@ -4744,14 +5010,14 @@
     </row>
     <row r="30" spans="1:4">
       <c r="A30" s="9" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B30" s="10"/>
       <c r="D30" s="10"/>
     </row>
     <row r="31" spans="1:4">
       <c r="A31" s="9" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B31" s="10" t="s">
         <v>24</v>
@@ -4760,7 +5026,7 @@
     </row>
     <row r="32" spans="1:4">
       <c r="A32" s="9" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B32" s="10" t="s">
         <v>24</v>
@@ -4769,7 +5035,7 @@
     </row>
     <row r="33" spans="1:4">
       <c r="A33" s="9" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B33" s="10" t="s">
         <v>24</v>
@@ -4778,7 +5044,7 @@
     </row>
     <row r="34" spans="1:4">
       <c r="A34" s="9" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B34" s="10" t="s">
         <v>24</v>
@@ -4787,10 +5053,10 @@
     </row>
     <row r="35" spans="1:4">
       <c r="A35" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="B35" s="10" t="s">
         <v>80</v>
-      </c>
-      <c r="B35" s="10" t="s">
-        <v>26</v>
       </c>
       <c r="D35" s="10"/>
     </row>
@@ -4843,7 +5109,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1786163787" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1786308497" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -4854,14 +5120,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1786163787" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1786163787" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1786308497" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1786308497" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1786163787" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1786308497" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -4880,7 +5146,7 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B1" s="11"/>
     </row>
@@ -4938,7 +5204,7 @@
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="9" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B9" s="10" t="s">
         <v>24</v>
@@ -5029,7 +5295,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1786163787" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1786308497" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -5040,14 +5306,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1786163787" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1786163787" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1786308497" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1786308497" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1786163787" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1786308497" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -5066,7 +5332,7 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B1" s="11"/>
     </row>
@@ -5119,7 +5385,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1786163787" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1786308497" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -5130,14 +5396,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1786163787" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1786163787" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1786308497" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1786308497" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1786163787" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1786308497" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -5156,7 +5422,7 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B1" s="11"/>
     </row>
@@ -5169,16 +5435,14 @@
         <v>104</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="9" t="s">
         <v>105</v>
       </c>
-      <c r="B4" s="10" t="s">
-        <v>26</v>
-      </c>
+      <c r="B4" s="10"/>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="9" t="s">
@@ -5272,16 +5536,14 @@
       <c r="A16" s="9" t="s">
         <v>117</v>
       </c>
-      <c r="B16" s="10" t="s">
-        <v>26</v>
-      </c>
+      <c r="B16" s="10"/>
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="9" t="s">
         <v>118</v>
       </c>
       <c r="B17" s="10" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="18" spans="1:2">
@@ -5289,7 +5551,7 @@
         <v>119</v>
       </c>
       <c r="B18" s="10" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="19" spans="1:2">
@@ -5297,7 +5559,7 @@
         <v>120</v>
       </c>
       <c r="B19" s="10" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="20" spans="1:2">
@@ -5305,7 +5567,7 @@
         <v>121</v>
       </c>
       <c r="B20" s="10" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="21" spans="1:2">
@@ -5521,7 +5783,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1786163787" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1786308497" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -5532,14 +5794,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1786163787" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1786163787" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1786308497" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1786308497" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1786163787" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1786308497" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -5558,7 +5820,7 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B1" s="11"/>
     </row>
@@ -5604,7 +5866,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1786163787" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1786308497" printRowHead="0" printColHead="0" printHeadLine="1" printFootLine="1" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -5615,14 +5877,14 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12&amp;KffffffPage &amp;P</oddFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1786163787" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1786163787" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1786308497" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1786308497" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1786163787" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1786308497" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>

</xml_diff>